<commit_message>
Bake Renovate 8 builder details into templates; add logo hook
- Add scripts/config.json with Renovate 8 ABN, licence, address, contact
- Update build_notice_template.py and build_register_template.py to read
  builder values from config.json and substitute into the generated
  templates (falls back to {{BUILDER_*}} placeholders if config absent)
- Add logo hook: if templates/logo.png (.jpg/.jpeg) exists it replaces
  the "RENOVATE 8" text heading on the notice
- README: document logo drop-in
</commit_message>
<xml_diff>
--- a/templates/master_register_template.xlsx
+++ b/templates/master_register_template.xlsx
@@ -3427,15 +3427,23 @@
           <t>Builder ABN</t>
         </is>
       </c>
-      <c r="B11" s="21" t="inlineStr"/>
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>72 098 695 446</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="20" t="inlineStr">
         <is>
-          <t>Builder NSW Contractor License #</t>
-        </is>
-      </c>
-      <c r="B12" s="21" t="inlineStr"/>
+          <t>Builder NSW Contractor Licence #</t>
+        </is>
+      </c>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>139701C</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="20" t="inlineStr">
@@ -3443,7 +3451,11 @@
           <t>Builder address</t>
         </is>
       </c>
-      <c r="B13" s="21" t="inlineStr"/>
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t>62 Budyan Road, Grays Point NSW 2232</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="20" t="inlineStr">
@@ -3451,7 +3463,11 @@
           <t>Builder contact email</t>
         </is>
       </c>
-      <c r="B14" s="21" t="inlineStr"/>
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>paul@renovate8.com.au</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="inlineStr">
@@ -3459,7 +3475,11 @@
           <t>Builder contact phone</t>
         </is>
       </c>
-      <c r="B15" s="21" t="inlineStr"/>
+      <c r="B15" s="21" t="inlineStr">
+        <is>
+          <t>0404 899 899</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="20" t="inlineStr">

</xml_diff>

<commit_message>
Add Renovate 8 logo + Gold and Eagle Constructions legal entity
- Extract logo from supplied Annandale quotation document and save as
  templates/logo.jpg (271x39 JPEG)
- Add the licence-holder entity ("Gold and Eagle Constructions trading
  as Renovate 8") to the notice header and footer, plus a dedicated
  "Builder legal entity (licence holder)" row in the register's
  Project Setup tab
- Update defined-name row references in the register to match the new
  Project Setup layout
</commit_message>
<xml_diff>
--- a/templates/master_register_template.xlsx
+++ b/templates/master_register_template.xlsx
@@ -23,8 +23,9 @@
     <definedName name="ClientName">'Project Setup'!$B$5</definedName>
     <definedName name="OriginalContractSum">'Project Setup'!$B$9</definedName>
     <definedName name="BuilderName">'Project Setup'!$B$10</definedName>
-    <definedName name="BuilderABN">'Project Setup'!$B$11</definedName>
-    <definedName name="BuilderLicense">'Project Setup'!$B$12</definedName>
+    <definedName name="BuilderLegalEntity">'Project Setup'!$B$11</definedName>
+    <definedName name="BuilderABN">'Project Setup'!$B$12</definedName>
+    <definedName name="BuilderLicense">'Project Setup'!$B$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3333,7 +3334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -3412,7 +3413,7 @@
     <row r="10">
       <c r="A10" s="20" t="inlineStr">
         <is>
-          <t>Builder name</t>
+          <t>Builder name (brand)</t>
         </is>
       </c>
       <c r="B10" s="21" t="inlineStr">
@@ -3424,90 +3425,102 @@
     <row r="11">
       <c r="A11" s="20" t="inlineStr">
         <is>
-          <t>Builder ABN</t>
+          <t>Builder legal entity (licence holder)</t>
         </is>
       </c>
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>72 098 695 446</t>
+          <t>Gold and Eagle Constructions</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="20" t="inlineStr">
         <is>
-          <t>Builder NSW Contractor Licence #</t>
+          <t>Builder ABN</t>
         </is>
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>139701C</t>
+          <t>72 098 695 446</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="20" t="inlineStr">
         <is>
-          <t>Builder address</t>
+          <t>Builder NSW Contractor Licence #</t>
         </is>
       </c>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>62 Budyan Road, Grays Point NSW 2232</t>
+          <t>139701C</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t>Builder contact email</t>
+          <t>Builder address</t>
         </is>
       </c>
       <c r="B14" s="21" t="inlineStr">
         <is>
-          <t>paul@renovate8.com.au</t>
+          <t>62 Budyan Road, Grays Point NSW 2232</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="inlineStr">
         <is>
-          <t>Builder contact phone</t>
+          <t>Builder contact email</t>
         </is>
       </c>
       <c r="B15" s="21" t="inlineStr">
         <is>
-          <t>0404 899 899</t>
+          <t>paul@renovate8.com.au</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="20" t="inlineStr">
         <is>
-          <t>Contract form</t>
+          <t>Builder contact phone</t>
         </is>
       </c>
       <c r="B16" s="21" t="inlineStr">
         <is>
-          <t>MBA NSW Residential Building Contract</t>
+          <t>0404 899 899</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="20" t="inlineStr">
         <is>
-          <t>Dropbox root for project</t>
-        </is>
-      </c>
-      <c r="B17" s="21" t="inlineStr"/>
+          <t>Contract form</t>
+        </is>
+      </c>
+      <c r="B17" s="21" t="inlineStr">
+        <is>
+          <t>MBA NSW Residential Building Contract</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
         <is>
+          <t>Dropbox root for project</t>
+        </is>
+      </c>
+      <c r="B18" s="21" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
           <t>Default markup %</t>
         </is>
       </c>
-      <c r="B18" s="21" t="inlineStr">
+      <c r="B19" s="21" t="inlineStr">
         <is>
           <t>(leave blank — set per variation)</t>
         </is>

</xml_diff>